<commit_message>
feat(import): nhập Excel = ghi đè toàn bộ qua 1 RPC, kèm danh mục + thứ tự menu
- bulk_import_menu: ghi cả plan trong 1 transaction thay vì ~1000 request lẻ
  (SECURITY INVOKER, RLS giữ nguyên). v2 thêm danh mục (is_divider) + xếp thứ tự,
  v3 ghi đè theo từng sheet có trong file: món/danh mục ngoài file → is_active=false,
  topping/tùy chọn/công thức/liên kết ngoài file → xoá. Nguyên liệu không xoá.
- Excel: cột "Danh mục" ở sheet Sản phẩm (xuất + nhập), xuất không còn biến dòng
  mục thành món 0đ. Xem trước liệt kê những gì sẽ bị xoá.
- sync_ingredient_key: bỏ dòng công thức old_key khi món đã có new_key
  (duplicate key idx_recipes_product_ingredient_address).
- KeySyncModal: làm mới ngay sau đồng bộ để banner cảnh báo tắt, reset khi đóng.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/mau-nhap-lieu.xlsx
+++ b/public/templates/mau-nhap-lieu.xlsx
@@ -405,7 +405,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -419,7 +419,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2. Sản phẩm/Nguyên liệu/Topping: trùng tên với dữ liệu đã có sẽ CẬP NHẬT giá (Nguyên liệu cập nhật cả đơn vị) — không tạo trùng.</v>
+        <v>2. Nhập = GHI ĐÈ TOÀN BỘ: sheet nào có trong file thì phần đó của địa chỉ được thay hoàn toàn theo file. Món, danh mục, topping, tùy chọn, công thức không có trong file sẽ bị XOÁ. Sheet nào xoá khỏi file thì phần đó giữ nguyên. Nguyên liệu không bao giờ bị xoá, chỉ thêm/cập nhật giá vốn và đơn vị.</v>
       </c>
     </row>
     <row r="4">
@@ -444,19 +444,24 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>7. Sheet Topping áp dụng món: ghi đè TOÀN BỘ danh sách món của mỗi topping trong file — món cũ không có trong file sẽ bị gỡ liên kết.</v>
+        <v>7. Sheet Topping áp dụng món: toàn bộ liên kết topping-món được thay theo file.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>8. Cột Danh mục (sheet Sản phẩm, tuỳ chọn): điền tên danh mục để nhóm món và xếp thứ tự menu đúng theo thứ tự dòng trong file. Danh mục chưa có sẽ được tạo mới. Để trống toàn bộ cột = không đổi thứ tự menu hiện tại.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A9"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:C3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -465,6 +470,9 @@
       <c r="B1" t="str">
         <v>Giá bán</v>
       </c>
+      <c r="C1" t="str">
+        <v>Danh mục</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -473,6 +481,9 @@
       <c r="B2">
         <v>16000</v>
       </c>
+      <c r="C2" t="str">
+        <v>Cà phê</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -481,10 +492,13 @@
       <c r="B3">
         <v>18000</v>
       </c>
+      <c r="C3" t="str">
+        <v>Cà phê</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C3"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>